<commit_message>
Auto rebuild Baltica figures, maps, and pages
</commit_message>
<xml_diff>
--- a/data/Baltica_paleolatitudes_64N_28E.xlsx
+++ b/data/Baltica_paleolatitudes_64N_28E.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y60"/>
+  <dimension ref="A1:Y59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,10 +575,10 @@
         <v>65.5</v>
       </c>
       <c r="I2" t="n">
-        <v>293</v>
+        <v>299.7</v>
       </c>
       <c r="J2" t="n">
-        <v>31.3</v>
+        <v>41.9</v>
       </c>
       <c r="K2" t="n">
         <v>9.9</v>
@@ -595,10 +595,10 @@
         <v>556</v>
       </c>
       <c r="O2" t="n">
-        <v>293</v>
+        <v>299.7</v>
       </c>
       <c r="P2" t="n">
-        <v>31.3</v>
+        <v>41.9</v>
       </c>
       <c r="Q2" t="n">
         <v>9.9</v>
@@ -621,13 +621,13 @@
         <v>28</v>
       </c>
       <c r="W2" t="n">
-        <v>25.74042619297266</v>
+        <v>37.58397653153573</v>
       </c>
       <c r="X2" t="n">
-        <v>289.0951494605843</v>
+        <v>290.1443272909424</v>
       </c>
       <c r="Y2" t="n">
-        <v>43.95801292576599</v>
+        <v>56.99067609882788</v>
       </c>
     </row>
     <row r="3">
@@ -662,10 +662,10 @@
         <v>58.5</v>
       </c>
       <c r="I3" t="n">
-        <v>306.7</v>
+        <v>308.1</v>
       </c>
       <c r="J3" t="n">
-        <v>17.3</v>
+        <v>19.7</v>
       </c>
       <c r="K3" t="n">
         <v>6</v>
@@ -682,10 +682,10 @@
         <v>570</v>
       </c>
       <c r="O3" t="n">
-        <v>306.7</v>
+        <v>308.1</v>
       </c>
       <c r="P3" t="n">
-        <v>17.3</v>
+        <v>19.7</v>
       </c>
       <c r="Q3" t="n">
         <v>6</v>
@@ -708,13 +708,13 @@
         <v>28</v>
       </c>
       <c r="W3" t="n">
-        <v>19.3044326047229</v>
+        <v>22.04628231378324</v>
       </c>
       <c r="X3" t="n">
-        <v>270.0339129930143</v>
+        <v>269.961649217816</v>
       </c>
       <c r="Y3" t="n">
-        <v>35.01369249445501</v>
+        <v>39.00513173055605</v>
       </c>
     </row>
     <row r="4">
@@ -725,7 +725,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Zigan formation clastic rocks -C</t>
+          <t>Zigan HTC thin beds</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -746,20 +746,20 @@
         <v>56.7</v>
       </c>
       <c r="H4" t="n">
-        <v>53.7</v>
+        <v>54.4</v>
       </c>
       <c r="I4" t="n">
-        <v>138.4</v>
+        <v>142.1</v>
       </c>
       <c r="J4" t="n">
-        <v>-16.2</v>
+        <v>-22.8</v>
       </c>
       <c r="K4" t="n">
-        <v>4.1</v>
+        <v>10.7</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Levashova, N.M., Bazhenov, M.L., Meert, J.G., Kuznetsov, N.B., Golovanova, I.V., Danukalov, K.N., Fedorova, N.M.</t>
+          <t>Bazhenov, M.L., Levashova, N.M., Meert, J.G., Golovanova, I.V., Danukalov, K.N., Fedorova, N.M.</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -769,13 +769,13 @@
         <v>571</v>
       </c>
       <c r="O4" t="n">
-        <v>138.4</v>
+        <v>142.1</v>
       </c>
       <c r="P4" t="n">
-        <v>-16.2</v>
+        <v>-22.8</v>
       </c>
       <c r="Q4" t="n">
-        <v>4.1</v>
+        <v>10.7</v>
       </c>
       <c r="R4" t="n">
         <v>5</v>
@@ -795,13 +795,13 @@
         <v>28</v>
       </c>
       <c r="W4" t="n">
-        <v>-23.42149663928187</v>
+        <v>-30.88459153588188</v>
       </c>
       <c r="X4" t="n">
-        <v>78.77946865560871</v>
+        <v>78.68017669899653</v>
       </c>
       <c r="Y4" t="n">
-        <v>-40.90461999354371</v>
+        <v>-50.10608937483194</v>
       </c>
     </row>
     <row r="5">
@@ -812,7 +812,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Zigan HTC thin beds</t>
+          <t>Zigan formation clastic rocks -C</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -833,20 +833,20 @@
         <v>56.7</v>
       </c>
       <c r="H5" t="n">
-        <v>54.4</v>
+        <v>53.7</v>
       </c>
       <c r="I5" t="n">
-        <v>138.3</v>
+        <v>140.2</v>
       </c>
       <c r="J5" t="n">
-        <v>-18</v>
+        <v>-20.8</v>
       </c>
       <c r="K5" t="n">
-        <v>10.7</v>
+        <v>4.1</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Bazhenov, M.L., Levashova, N.M., Meert, J.G., Golovanova, I.V., Danukalov, K.N., Fedorova, N.M.</t>
+          <t>Levashova, N.M., Bazhenov, M.L., Meert, J.G., Kuznetsov, N.B., Golovanova, I.V., Danukalov, K.N., Fedorova, N.M.</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -856,13 +856,13 @@
         <v>571</v>
       </c>
       <c r="O5" t="n">
-        <v>138.3</v>
+        <v>140.2</v>
       </c>
       <c r="P5" t="n">
-        <v>-18</v>
+        <v>-20.8</v>
       </c>
       <c r="Q5" t="n">
-        <v>10.7</v>
+        <v>4.1</v>
       </c>
       <c r="R5" t="n">
         <v>5</v>
@@ -882,13 +882,13 @@
         <v>28</v>
       </c>
       <c r="W5" t="n">
-        <v>-24.98529018596297</v>
+        <v>-28.29474200208585</v>
       </c>
       <c r="X5" t="n">
-        <v>79.76240362140653</v>
+        <v>79.41150972849623</v>
       </c>
       <c r="Y5" t="n">
-        <v>-42.98391218087836</v>
+        <v>-47.11391226811408</v>
       </c>
     </row>
     <row r="6">
@@ -1010,10 +1010,10 @@
         <v>53.9</v>
       </c>
       <c r="I7" t="n">
-        <v>186.1</v>
+        <v>190.8</v>
       </c>
       <c r="J7" t="n">
-        <v>1.7</v>
+        <v>-7</v>
       </c>
       <c r="K7" t="n">
         <v>3.8</v>
@@ -1030,10 +1030,10 @@
         <v>575</v>
       </c>
       <c r="O7" t="n">
-        <v>186.1</v>
+        <v>190.8</v>
       </c>
       <c r="P7" t="n">
-        <v>1.7</v>
+        <v>-7</v>
       </c>
       <c r="Q7" t="n">
         <v>3.8</v>
@@ -1056,13 +1056,13 @@
         <v>28</v>
       </c>
       <c r="W7" t="n">
-        <v>-22.32710318402263</v>
+        <v>-31.68039451955769</v>
       </c>
       <c r="X7" t="n">
-        <v>23.76832627013995</v>
+        <v>20.17548619299581</v>
       </c>
       <c r="Y7" t="n">
-        <v>-39.39849289138143</v>
+        <v>-50.98599076316423</v>
       </c>
     </row>
     <row r="8">
@@ -1097,10 +1097,10 @@
         <v>54</v>
       </c>
       <c r="I8" t="n">
-        <v>187.3</v>
+        <v>192.4</v>
       </c>
       <c r="J8" t="n">
-        <v>1.1</v>
+        <v>-8.6</v>
       </c>
       <c r="K8" t="n">
         <v>5.8</v>
@@ -1117,10 +1117,10 @@
         <v>575</v>
       </c>
       <c r="O8" t="n">
-        <v>187.3</v>
+        <v>192.4</v>
       </c>
       <c r="P8" t="n">
-        <v>1.1</v>
+        <v>-8.6</v>
       </c>
       <c r="Q8" t="n">
         <v>5.8</v>
@@ -1143,13 +1143,13 @@
         <v>28</v>
       </c>
       <c r="W8" t="n">
-        <v>-23.12519483601076</v>
+        <v>-33.49586785608633</v>
       </c>
       <c r="X8" t="n">
-        <v>22.599523409567</v>
+        <v>18.59331974141105</v>
       </c>
       <c r="Y8" t="n">
-        <v>-40.50103598937987</v>
+        <v>-52.92764067834125</v>
       </c>
     </row>
     <row r="9">
@@ -1271,10 +1271,10 @@
         <v>54.94</v>
       </c>
       <c r="I10" t="n">
-        <v>299.1</v>
+        <v>308.8</v>
       </c>
       <c r="J10" t="n">
-        <v>42.3</v>
+        <v>51.5</v>
       </c>
       <c r="K10" t="n">
         <v>5.9</v>
@@ -1291,10 +1291,10 @@
         <v>650</v>
       </c>
       <c r="O10" t="n">
-        <v>299.1</v>
+        <v>308.8</v>
       </c>
       <c r="P10" t="n">
-        <v>42.3</v>
+        <v>51.5</v>
       </c>
       <c r="Q10" t="n">
         <v>5.9</v>
@@ -1317,13 +1317,13 @@
         <v>28</v>
       </c>
       <c r="W10" t="n">
-        <v>37.67082595540556</v>
+        <v>48.98506115356787</v>
       </c>
       <c r="X10" t="n">
-        <v>290.8919979641753</v>
+        <v>291.2854699569432</v>
       </c>
       <c r="Y10" t="n">
-        <v>57.07267844402786</v>
+        <v>66.49711257416338</v>
       </c>
     </row>
     <row r="11">
@@ -1358,10 +1358,10 @@
         <v>53.32</v>
       </c>
       <c r="I11" t="n">
-        <v>314.5</v>
+        <v>334.2</v>
       </c>
       <c r="J11" t="n">
-        <v>50.9</v>
+        <v>59.8</v>
       </c>
       <c r="K11" t="n">
         <v>5.3</v>
@@ -1378,10 +1378,10 @@
         <v>720</v>
       </c>
       <c r="O11" t="n">
-        <v>314.5</v>
+        <v>334.2</v>
       </c>
       <c r="P11" t="n">
-        <v>50.9</v>
+        <v>59.8</v>
       </c>
       <c r="Q11" t="n">
         <v>5.3</v>
@@ -1404,13 +1404,13 @@
         <v>28</v>
       </c>
       <c r="W11" t="n">
-        <v>50.89829457956896</v>
+        <v>65.09934023763316</v>
       </c>
       <c r="X11" t="n">
-        <v>286.5070826596683</v>
+        <v>285.4059580204532</v>
       </c>
       <c r="Y11" t="n">
-        <v>67.88496068234129</v>
+        <v>76.93305174232316</v>
       </c>
     </row>
     <row r="12">
@@ -1532,10 +1532,10 @@
         <v>54.5</v>
       </c>
       <c r="I13" t="n">
-        <v>171.7</v>
+        <v>164.6</v>
       </c>
       <c r="J13" t="n">
-        <v>35.8</v>
+        <v>43.7</v>
       </c>
       <c r="K13" t="n">
         <v>6.9</v>
@@ -1552,10 +1552,10 @@
         <v>1000</v>
       </c>
       <c r="O13" t="n">
-        <v>171.7</v>
+        <v>164.6</v>
       </c>
       <c r="P13" t="n">
-        <v>35.8</v>
+        <v>43.7</v>
       </c>
       <c r="Q13" t="n">
         <v>6.9</v>
@@ -1578,13 +1578,13 @@
         <v>28</v>
       </c>
       <c r="W13" t="n">
-        <v>13.8399842213621</v>
+        <v>22.99738938349144</v>
       </c>
       <c r="X13" t="n">
-        <v>29.63793936963697</v>
+        <v>32.65845903368475</v>
       </c>
       <c r="Y13" t="n">
-        <v>26.23072582414833</v>
+        <v>40.32599873916713</v>
       </c>
     </row>
     <row r="14">
@@ -3509,11 +3509,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Häme + E-W Satakunta</t>
+          <t>Häme dyke swarm</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1642</v>
+        <v>1647</v>
       </c>
       <c r="D36" t="n">
         <v>1633</v>
@@ -3523,27 +3523,27 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>24</v>
+        <v>25.1</v>
       </c>
       <c r="H36" t="n">
-        <v>61</v>
+        <v>61.4</v>
       </c>
       <c r="I36" t="n">
-        <v>209.1</v>
+        <v>209.8</v>
       </c>
       <c r="J36" t="n">
-        <v>26.3</v>
+        <v>23.6</v>
       </c>
       <c r="K36" t="n">
-        <v>10.9</v>
+        <v>14.7</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Salminen, J., Elming, S-Å, Mertanen, S., Almqvist, B., Wang, C., Moakhar, M.,</t>
+          <t>Salminen, J., Klein, R., Veikkolainen, T., Mertanen, S., Mänttäri, I.</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3553,19 +3553,19 @@
         <v>1661</v>
       </c>
       <c r="O36" t="n">
-        <v>209.1</v>
+        <v>209.8</v>
       </c>
       <c r="P36" t="n">
-        <v>26.3</v>
+        <v>23.6</v>
       </c>
       <c r="Q36" t="n">
-        <v>10.9</v>
+        <v>14.7</v>
       </c>
       <c r="R36" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="S36" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
@@ -3579,13 +3579,13 @@
         <v>28</v>
       </c>
       <c r="W36" t="n">
-        <v>0.3041496466790932</v>
+        <v>-2.388633013197776</v>
       </c>
       <c r="X36" t="n">
-        <v>359.0138629247815</v>
+        <v>358.3491558035057</v>
       </c>
       <c r="Y36" t="n">
-        <v>0.6082821529087816</v>
+        <v>-4.768991808099199</v>
       </c>
     </row>
     <row r="37">
@@ -3596,63 +3596,63 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Häme dyke swarm</t>
+          <t>Turinge gabbro-diabase</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1647</v>
+        <v>1700</v>
       </c>
       <c r="D37" t="n">
-        <v>1633</v>
+        <v>1696</v>
       </c>
       <c r="E37" t="n">
-        <v>1661</v>
+        <v>1704</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>25.1</v>
+        <v>15</v>
       </c>
       <c r="H37" t="n">
-        <v>61.4</v>
+        <v>63</v>
       </c>
       <c r="I37" t="n">
-        <v>209.8</v>
+        <v>220.2</v>
       </c>
       <c r="J37" t="n">
-        <v>23.6</v>
+        <v>51.6</v>
       </c>
       <c r="K37" t="n">
-        <v>14.7</v>
+        <v>4.8</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Salminen, J., Klein, R., Veikkolainen, T., Mertanen, S., Mänttäri, I.</t>
+          <t>Elming, Layer, Söderlund</t>
         </is>
       </c>
       <c r="M37" t="n">
-        <v>1633</v>
+        <v>1696</v>
       </c>
       <c r="N37" t="n">
-        <v>1661</v>
+        <v>1704</v>
       </c>
       <c r="O37" t="n">
-        <v>209.8</v>
+        <v>220.2</v>
       </c>
       <c r="P37" t="n">
-        <v>23.6</v>
+        <v>51.6</v>
       </c>
       <c r="Q37" t="n">
-        <v>14.7</v>
+        <v>4.8</v>
       </c>
       <c r="R37" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="S37" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="T37" t="inlineStr">
         <is>
@@ -3666,80 +3666,80 @@
         <v>28</v>
       </c>
       <c r="W37" t="n">
-        <v>-2.388633013197776</v>
+        <v>25.99133716878819</v>
       </c>
       <c r="X37" t="n">
-        <v>358.3491558035057</v>
+        <v>351.6028549862914</v>
       </c>
       <c r="Y37" t="n">
-        <v>-4.768991808099199</v>
+        <v>44.27744504374255</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Baltica</t>
+          <t>Baltica-Sarmatia</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Turinge gabbro-diabase</t>
+          <t>Volyn-Dniestr-Bug intrusions E</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1700</v>
+        <v>1722</v>
       </c>
       <c r="D38" t="n">
-        <v>1696</v>
+        <v>1710</v>
       </c>
       <c r="E38" t="n">
-        <v>1704</v>
+        <v>1734</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>15</v>
+        <v>29.6</v>
       </c>
       <c r="H38" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="I38" t="n">
-        <v>220.2</v>
+        <v>163.2</v>
       </c>
       <c r="J38" t="n">
-        <v>51.6</v>
+        <v>10.7</v>
       </c>
       <c r="K38" t="n">
-        <v>4.8</v>
+        <v>10.2</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Elming, Layer, Söderlund</t>
+          <t>Elming, S.-Ã…., Shumlyanskyy, L., Kravchenko, S., Layer, P., SÃ¶derlund, U.</t>
         </is>
       </c>
       <c r="M38" t="n">
-        <v>1696</v>
+        <v>1710</v>
       </c>
       <c r="N38" t="n">
-        <v>1704</v>
+        <v>1734</v>
       </c>
       <c r="O38" t="n">
-        <v>220.2</v>
+        <v>163.2</v>
       </c>
       <c r="P38" t="n">
-        <v>51.6</v>
+        <v>10.7</v>
       </c>
       <c r="Q38" t="n">
-        <v>4.8</v>
+        <v>10.2</v>
       </c>
       <c r="R38" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="S38" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="T38" t="inlineStr">
         <is>
@@ -3753,13 +3753,13 @@
         <v>28</v>
       </c>
       <c r="W38" t="n">
-        <v>25.99133716878819</v>
+        <v>-7.976730154751991</v>
       </c>
       <c r="X38" t="n">
-        <v>351.6028549862914</v>
+        <v>44.35862235901306</v>
       </c>
       <c r="Y38" t="n">
-        <v>44.27744504374255</v>
+        <v>-15.65570891331447</v>
       </c>
     </row>
     <row r="39">
@@ -3852,68 +3852,68 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Baltica</t>
+          <t>Baltica-Sarmatia</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Shoksha Sandstones</t>
+          <t>Volyn-Dniestr-Bug intrusions C+D</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1775</v>
+        <v>1755</v>
       </c>
       <c r="D40" t="n">
-        <v>1750</v>
+        <v>1740</v>
       </c>
       <c r="E40" t="n">
-        <v>1800</v>
+        <v>1770</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>33.799999</v>
+        <v>28.6</v>
       </c>
       <c r="H40" t="n">
-        <v>61.299999</v>
+        <v>50.6</v>
       </c>
       <c r="I40" t="n">
-        <v>221.100006</v>
+        <v>169.1</v>
       </c>
       <c r="J40" t="n">
-        <v>39.700001</v>
+        <v>26.5</v>
       </c>
       <c r="K40" t="n">
-        <v>3.99374511</v>
+        <v>3.9</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Pisarevsky, S.A., Sokolov, S.J.</t>
+          <t>Elming, S.-Ã…., Shumlyanskyy, L., Kravchenko, S., Layer, P., SÃ¶derlund, U.</t>
         </is>
       </c>
       <c r="M40" t="n">
-        <v>1750</v>
+        <v>1740</v>
       </c>
       <c r="N40" t="n">
-        <v>1800</v>
+        <v>1770</v>
       </c>
       <c r="O40" t="n">
-        <v>221.100006</v>
+        <v>169.1</v>
       </c>
       <c r="P40" t="n">
-        <v>39.700001</v>
+        <v>26.5</v>
       </c>
       <c r="Q40" t="n">
-        <v>3.99374511</v>
+        <v>3.9</v>
       </c>
       <c r="R40" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="S40" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="T40" t="inlineStr">
         <is>
@@ -3927,13 +3927,13 @@
         <v>28</v>
       </c>
       <c r="W40" t="n">
-        <v>14.21821806742281</v>
+        <v>5.493033338051561</v>
       </c>
       <c r="X40" t="n">
-        <v>349.6362863668787</v>
+        <v>34.37301626167139</v>
       </c>
       <c r="Y40" t="n">
-        <v>26.87381764398741</v>
+        <v>10.88690669551862</v>
       </c>
     </row>
     <row r="41">
@@ -3944,17 +3944,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Småland intrusives -C</t>
+          <t>Shoksha Sandstones</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1776.5</v>
+        <v>1775</v>
       </c>
       <c r="D41" t="n">
-        <v>1769</v>
+        <v>1750</v>
       </c>
       <c r="E41" t="n">
-        <v>1784</v>
+        <v>1800</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -3962,45 +3962,45 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>15.7</v>
+        <v>33.799999</v>
       </c>
       <c r="H41" t="n">
-        <v>57.1</v>
+        <v>61.299999</v>
       </c>
       <c r="I41" t="n">
-        <v>182.7</v>
+        <v>221.7</v>
       </c>
       <c r="J41" t="n">
-        <v>45.7</v>
+        <v>46.8</v>
       </c>
       <c r="K41" t="n">
-        <v>8</v>
+        <v>3.99374511</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Pisarevsky, S., Bylund, G.</t>
+          <t>Pisarevsky, S.A., Sokolov, S.J.</t>
         </is>
       </c>
       <c r="M41" t="n">
-        <v>1769</v>
+        <v>1750</v>
       </c>
       <c r="N41" t="n">
-        <v>1784</v>
+        <v>1800</v>
       </c>
       <c r="O41" t="n">
-        <v>182.7</v>
+        <v>221.7</v>
       </c>
       <c r="P41" t="n">
-        <v>45.7</v>
+        <v>46.8</v>
       </c>
       <c r="Q41" t="n">
-        <v>8</v>
+        <v>3.99374511</v>
       </c>
       <c r="R41" t="n">
-        <v>7.5</v>
+        <v>25</v>
       </c>
       <c r="S41" t="n">
-        <v>7.5</v>
+        <v>25</v>
       </c>
       <c r="T41" t="inlineStr">
         <is>
@@ -4014,13 +4014,13 @@
         <v>28</v>
       </c>
       <c r="W41" t="n">
-        <v>21.4975742570288</v>
+        <v>21.32419682997836</v>
       </c>
       <c r="X41" t="n">
-        <v>18.7106837385896</v>
+        <v>349.9770757235874</v>
       </c>
       <c r="Y41" t="n">
-        <v>38.22832239799614</v>
+        <v>37.98060354714293</v>
       </c>
     </row>
     <row r="42">
@@ -4031,63 +4031,63 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Hoting gabbro</t>
+          <t>Småland intrusives -C</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1786</v>
+        <v>1776.5</v>
       </c>
       <c r="D42" t="n">
-        <v>1776</v>
+        <v>1769</v>
       </c>
       <c r="E42" t="n">
-        <v>1796</v>
+        <v>1784</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>16.2</v>
+        <v>15.7</v>
       </c>
       <c r="H42" t="n">
-        <v>64.2</v>
+        <v>57.1</v>
       </c>
       <c r="I42" t="n">
-        <v>233.3</v>
+        <v>182.7</v>
       </c>
       <c r="J42" t="n">
-        <v>43</v>
+        <v>45.7</v>
       </c>
       <c r="K42" t="n">
-        <v>10.9</v>
+        <v>8</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Elming, S.Å., Moakhar, M.O., Layer, P and Donadini, F.</t>
+          <t>Pisarevsky, S., Bylund, G.</t>
         </is>
       </c>
       <c r="M42" t="n">
-        <v>1776</v>
+        <v>1769</v>
       </c>
       <c r="N42" t="n">
-        <v>1796</v>
+        <v>1784</v>
       </c>
       <c r="O42" t="n">
-        <v>233.3</v>
+        <v>182.7</v>
       </c>
       <c r="P42" t="n">
-        <v>43</v>
+        <v>45.7</v>
       </c>
       <c r="Q42" t="n">
-        <v>10.9</v>
+        <v>8</v>
       </c>
       <c r="R42" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="S42" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="T42" t="inlineStr">
         <is>
@@ -4101,80 +4101,80 @@
         <v>28</v>
       </c>
       <c r="W42" t="n">
-        <v>18.85191182326832</v>
+        <v>21.4975742570288</v>
       </c>
       <c r="X42" t="n">
-        <v>340.7150624909892</v>
+        <v>18.7106837385896</v>
       </c>
       <c r="Y42" t="n">
-        <v>34.32831817390197</v>
+        <v>38.22832239799614</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Baltica-Fennoscandia</t>
+          <t>Baltica</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Lake Ladoga/ Mean intr. &amp; dykes/ A</t>
+          <t>Hoting gabbro</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1800</v>
+        <v>1786</v>
       </c>
       <c r="D43" t="n">
-        <v>1744</v>
+        <v>1776</v>
       </c>
       <c r="E43" t="n">
-        <v>1819</v>
+        <v>1796</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>30</v>
+        <v>16.2</v>
       </c>
       <c r="H43" t="n">
-        <v>61.3</v>
+        <v>64.2</v>
       </c>
       <c r="I43" t="n">
-        <v>229.1</v>
+        <v>233.3</v>
       </c>
       <c r="J43" t="n">
-        <v>50.9</v>
+        <v>43</v>
       </c>
       <c r="K43" t="n">
-        <v>7.2</v>
+        <v>10.9</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Mertanen, S., Eklund, O., Shebanov, A., Frank-Kamenetsky, D.</t>
+          <t>Elming, S.Å., Moakhar, M.O., Layer, P and Donadini, F.</t>
         </is>
       </c>
       <c r="M43" t="n">
-        <v>1744</v>
+        <v>1776</v>
       </c>
       <c r="N43" t="n">
-        <v>1819</v>
+        <v>1796</v>
       </c>
       <c r="O43" t="n">
-        <v>229.1</v>
+        <v>233.3</v>
       </c>
       <c r="P43" t="n">
-        <v>50.9</v>
+        <v>43</v>
       </c>
       <c r="Q43" t="n">
-        <v>7.2</v>
+        <v>10.9</v>
       </c>
       <c r="R43" t="n">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="S43" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="T43" t="inlineStr">
         <is>
@@ -4188,13 +4188,13 @@
         <v>28</v>
       </c>
       <c r="W43" t="n">
-        <v>26.07658611736225</v>
+        <v>18.85191182326832</v>
       </c>
       <c r="X43" t="n">
-        <v>345.3584189143534</v>
+        <v>340.7150624909892</v>
       </c>
       <c r="Y43" t="n">
-        <v>44.38549807829641</v>
+        <v>34.32831817390197</v>
       </c>
     </row>
     <row r="44">
@@ -4205,63 +4205,63 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Notträsk gabbro</t>
+          <t>Lake Ladoga/ Mean intr. &amp; dykes/ A</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1806</v>
+        <v>1800</v>
       </c>
       <c r="D44" t="n">
-        <v>1800</v>
+        <v>1744</v>
       </c>
       <c r="E44" t="n">
-        <v>1812</v>
+        <v>1819</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>21.83</v>
+        <v>30</v>
       </c>
       <c r="H44" t="n">
-        <v>65.83</v>
+        <v>61.3</v>
       </c>
       <c r="I44" t="n">
-        <v>216.2</v>
+        <v>229.1</v>
       </c>
       <c r="J44" t="n">
-        <v>43.5</v>
+        <v>50.9</v>
       </c>
       <c r="K44" t="n">
-        <v>6.1</v>
+        <v>7.2</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Elming</t>
+          <t>Mertanen, S., Eklund, O., Shebanov, A., Frank-Kamenetsky, D.</t>
         </is>
       </c>
       <c r="M44" t="n">
-        <v>1800</v>
+        <v>1744</v>
       </c>
       <c r="N44" t="n">
-        <v>1812</v>
+        <v>1819</v>
       </c>
       <c r="O44" t="n">
-        <v>216.2</v>
+        <v>229.1</v>
       </c>
       <c r="P44" t="n">
-        <v>43.5</v>
+        <v>50.9</v>
       </c>
       <c r="Q44" t="n">
-        <v>6.1</v>
+        <v>7.2</v>
       </c>
       <c r="R44" t="n">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="S44" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="T44" t="inlineStr">
         <is>
@@ -4275,13 +4275,13 @@
         <v>28</v>
       </c>
       <c r="W44" t="n">
-        <v>17.69541268283204</v>
+        <v>26.07658611736225</v>
       </c>
       <c r="X44" t="n">
-        <v>353.7655215751807</v>
+        <v>345.3584189143534</v>
       </c>
       <c r="Y44" t="n">
-        <v>32.54215048836207</v>
+        <v>44.38549807829641</v>
       </c>
     </row>
     <row r="45">
@@ -4292,63 +4292,63 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Eastern Murmansk sills</t>
+          <t>Notträsk gabbro</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1860</v>
+        <v>1806</v>
       </c>
       <c r="D45" t="n">
-        <v>1856</v>
+        <v>1800</v>
       </c>
       <c r="E45" t="n">
-        <v>1870</v>
+        <v>1812</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="G45" t="n">
-        <v>38.2</v>
+        <v>21.83</v>
       </c>
       <c r="H45" t="n">
-        <v>68.5</v>
+        <v>65.83</v>
       </c>
       <c r="I45" t="n">
-        <v>234.7</v>
+        <v>216.2</v>
       </c>
       <c r="J45" t="n">
-        <v>54.7</v>
+        <v>43.5</v>
       </c>
       <c r="K45" t="n">
-        <v>5.2</v>
+        <v>6.1</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Veselovskiy et al.</t>
+          <t>Elming</t>
         </is>
       </c>
       <c r="M45" t="n">
-        <v>1856</v>
+        <v>1800</v>
       </c>
       <c r="N45" t="n">
-        <v>1870</v>
+        <v>1812</v>
       </c>
       <c r="O45" t="n">
-        <v>234.7</v>
+        <v>216.2</v>
       </c>
       <c r="P45" t="n">
-        <v>54.7</v>
+        <v>43.5</v>
       </c>
       <c r="Q45" t="n">
-        <v>5.2</v>
+        <v>6.1</v>
       </c>
       <c r="R45" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S45" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="T45" t="inlineStr">
         <is>
@@ -4362,13 +4362,13 @@
         <v>28</v>
       </c>
       <c r="W45" t="n">
-        <v>30.47977899500718</v>
+        <v>17.69541268283204</v>
       </c>
       <c r="X45" t="n">
-        <v>342.4657221886084</v>
+        <v>353.7655215751807</v>
       </c>
       <c r="Y45" t="n">
-        <v>49.65153320146266</v>
+        <v>32.54215048836207</v>
       </c>
     </row>
     <row r="46">
@@ -4379,17 +4379,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Keuruu dykes</t>
+          <t>Eastern Murmansk sills</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1869</v>
+        <v>1860</v>
       </c>
       <c r="D46" t="n">
-        <v>1859</v>
+        <v>1856</v>
       </c>
       <c r="E46" t="n">
-        <v>1879</v>
+        <v>1870</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -4397,42 +4397,42 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>24.7</v>
+        <v>38.2</v>
       </c>
       <c r="H46" t="n">
-        <v>62.3</v>
+        <v>68.5</v>
       </c>
       <c r="I46" t="n">
-        <v>230.9</v>
+        <v>234.7</v>
       </c>
       <c r="J46" t="n">
-        <v>45.7</v>
+        <v>54.7</v>
       </c>
       <c r="K46" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Klein, R., Pesonen, L.J., Mänttäri, I., Heinonen, J.S.</t>
+          <t>Veselovskiy et al.</t>
         </is>
       </c>
       <c r="M46" t="n">
-        <v>1859</v>
+        <v>1856</v>
       </c>
       <c r="N46" t="n">
-        <v>1879</v>
+        <v>1870</v>
       </c>
       <c r="O46" t="n">
-        <v>230.9</v>
+        <v>234.7</v>
       </c>
       <c r="P46" t="n">
-        <v>45.7</v>
+        <v>54.7</v>
       </c>
       <c r="Q46" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
       <c r="R46" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="S46" t="n">
         <v>10</v>
@@ -4449,13 +4449,13 @@
         <v>28</v>
       </c>
       <c r="W46" t="n">
-        <v>21.17547955578922</v>
+        <v>30.47977899500718</v>
       </c>
       <c r="X46" t="n">
-        <v>343.0552620149157</v>
+        <v>342.4657221886084</v>
       </c>
       <c r="Y46" t="n">
-        <v>37.76724778186111</v>
+        <v>49.65153320146266</v>
       </c>
     </row>
     <row r="47">
@@ -4466,17 +4466,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Svecofennian gabbro intrusions</t>
+          <t>Keuruu dykes</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1885</v>
+        <v>1869</v>
       </c>
       <c r="D47" t="n">
-        <v>1875</v>
+        <v>1859</v>
       </c>
       <c r="E47" t="n">
-        <v>1891</v>
+        <v>1879</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -4484,45 +4484,45 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>25.08</v>
+        <v>24.7</v>
       </c>
       <c r="H47" t="n">
-        <v>63.9</v>
+        <v>62.3</v>
       </c>
       <c r="I47" t="n">
-        <v>237.5</v>
+        <v>230.9</v>
       </c>
       <c r="J47" t="n">
-        <v>46.9</v>
+        <v>45.7</v>
       </c>
       <c r="K47" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Luoto, T., Salminen, J., Mertanen, S., Elming, S.-Å-, Pesonen, L.J.</t>
+          <t>Klein, R., Pesonen, L.J., Mänttäri, I., Heinonen, J.S.</t>
         </is>
       </c>
       <c r="M47" t="n">
-        <v>1875</v>
+        <v>1859</v>
       </c>
       <c r="N47" t="n">
-        <v>1891</v>
+        <v>1879</v>
       </c>
       <c r="O47" t="n">
-        <v>237.5</v>
+        <v>230.9</v>
       </c>
       <c r="P47" t="n">
-        <v>46.9</v>
+        <v>45.7</v>
       </c>
       <c r="Q47" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="R47" t="n">
         <v>10</v>
       </c>
       <c r="S47" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="T47" t="inlineStr">
         <is>
@@ -4536,80 +4536,80 @@
         <v>28</v>
       </c>
       <c r="W47" t="n">
-        <v>23.30153040037972</v>
+        <v>21.17547955578922</v>
       </c>
       <c r="X47" t="n">
-        <v>338.5099061673419</v>
+        <v>343.0552620149157</v>
       </c>
       <c r="Y47" t="n">
-        <v>40.74159036254147</v>
+        <v>37.76724778186111</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Baltica-Karelia</t>
+          <t>Baltica-Fennoscandia</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Onega 1975 Ma Intrusions</t>
+          <t>Svecofennian gabbro intrusions</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1976</v>
+        <v>1885</v>
       </c>
       <c r="D48" t="n">
-        <v>1967</v>
+        <v>1875</v>
       </c>
       <c r="E48" t="n">
-        <v>1985</v>
+        <v>1891</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>34</v>
+        <v>25.08</v>
       </c>
       <c r="H48" t="n">
-        <v>62.1</v>
+        <v>63.9</v>
       </c>
       <c r="I48" t="n">
-        <v>101.5</v>
+        <v>237.5</v>
       </c>
       <c r="J48" t="n">
-        <v>44.4</v>
+        <v>46.9</v>
       </c>
       <c r="K48" t="n">
-        <v>6.3</v>
+        <v>3.5</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Lubnina, N.V., Pisarevsky, S.A., Stepanova, A.V., Bogdanova, S.V., Sokolov, S.J.</t>
+          <t>Luoto, T., Salminen, J., Mertanen, S., Elming, S.-Å-, Pesonen, L.J.</t>
         </is>
       </c>
       <c r="M48" t="n">
-        <v>1967</v>
+        <v>1875</v>
       </c>
       <c r="N48" t="n">
-        <v>1985</v>
+        <v>1891</v>
       </c>
       <c r="O48" t="n">
-        <v>101.5</v>
+        <v>237.5</v>
       </c>
       <c r="P48" t="n">
-        <v>44.4</v>
+        <v>46.9</v>
       </c>
       <c r="Q48" t="n">
-        <v>6.3</v>
+        <v>3.5</v>
       </c>
       <c r="R48" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S48" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="T48" t="inlineStr">
         <is>
@@ -4623,34 +4623,34 @@
         <v>28</v>
       </c>
       <c r="W48" t="n">
-        <v>45.87380392146377</v>
+        <v>23.30153040037972</v>
       </c>
       <c r="X48" t="n">
-        <v>79.71351546234041</v>
+        <v>338.5099061673419</v>
       </c>
       <c r="Y48" t="n">
-        <v>64.12767286642595</v>
+        <v>40.74159036254147</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Baltica-Karelia</t>
+          <t>Baltica-Kola</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Varpaisjärvi dolerites &amp; basement</t>
+          <t>Tsuomasvarri Gabbro-Diorite Intrusion</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2295</v>
+        <v>1931</v>
       </c>
       <c r="D49" t="n">
-        <v>2290</v>
+        <v>1929</v>
       </c>
       <c r="E49" t="n">
-        <v>2300</v>
+        <v>1933</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -4658,45 +4658,45 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>27.8</v>
+        <v>28.299999</v>
       </c>
       <c r="H49" t="n">
-        <v>63.4</v>
+        <v>69.900002</v>
       </c>
       <c r="I49" t="n">
-        <v>262.3</v>
+        <v>247.300003</v>
       </c>
       <c r="J49" t="n">
-        <v>-17.4</v>
+        <v>40.200001</v>
       </c>
       <c r="K49" t="n">
-        <v>9.800000000000001</v>
+        <v>6.015812497</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Mertanen, S., Hölttä, P., Pesonen, L.J., Paavola, J.,</t>
+          <t>Mertanen,S., Pesonen,L.J.</t>
         </is>
       </c>
       <c r="M49" t="n">
-        <v>2290</v>
+        <v>1929</v>
       </c>
       <c r="N49" t="n">
-        <v>2300</v>
+        <v>1933</v>
       </c>
       <c r="O49" t="n">
-        <v>262.3</v>
+        <v>247.300003</v>
       </c>
       <c r="P49" t="n">
-        <v>-17.4</v>
+        <v>40.200001</v>
       </c>
       <c r="Q49" t="n">
-        <v>9.800000000000001</v>
+        <v>6.015812497</v>
       </c>
       <c r="R49" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S49" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T49" t="inlineStr">
         <is>
@@ -4710,13 +4710,13 @@
         <v>28</v>
       </c>
       <c r="W49" t="n">
-        <v>-30.85572545050428</v>
+        <v>18.72532451752087</v>
       </c>
       <c r="X49" t="n">
-        <v>295.4863304832984</v>
+        <v>329.2820768653556</v>
       </c>
       <c r="Y49" t="n">
-        <v>-50.07383311007023</v>
+        <v>34.13523227034082</v>
       </c>
     </row>
     <row r="50">
@@ -4727,63 +4727,63 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Taivalkoski 2.3 Ga dyke</t>
+          <t>Onega 1975 Ma Intrusions</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2339</v>
+        <v>1976</v>
       </c>
       <c r="D50" t="n">
-        <v>2321</v>
+        <v>1967</v>
       </c>
       <c r="E50" t="n">
-        <v>2357</v>
+        <v>1985</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>28.1</v>
+        <v>34</v>
       </c>
       <c r="H50" t="n">
-        <v>65.5</v>
+        <v>62.1</v>
       </c>
       <c r="I50" t="n">
-        <v>257.3</v>
+        <v>101.5</v>
       </c>
       <c r="J50" t="n">
-        <v>20.4</v>
+        <v>44.4</v>
       </c>
       <c r="K50" t="n">
         <v>6.3</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Salminen, J., Halls, H.C., Mertanen, S., Pesonen, L.J., Vuollo, J., SÃ¶derlund, U.</t>
+          <t>Lubnina, N.V., Pisarevsky, S.A., Stepanova, A.V., Bogdanova, S.V., Sokolov, S.J.</t>
         </is>
       </c>
       <c r="M50" t="n">
-        <v>2321</v>
+        <v>1967</v>
       </c>
       <c r="N50" t="n">
-        <v>2357</v>
+        <v>1985</v>
       </c>
       <c r="O50" t="n">
-        <v>257.3</v>
+        <v>101.5</v>
       </c>
       <c r="P50" t="n">
-        <v>20.4</v>
+        <v>44.4</v>
       </c>
       <c r="Q50" t="n">
         <v>6.3</v>
       </c>
       <c r="R50" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="S50" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="T50" t="inlineStr">
         <is>
@@ -4797,34 +4797,34 @@
         <v>28</v>
       </c>
       <c r="W50" t="n">
-        <v>2.599943141397745</v>
+        <v>45.87380392146377</v>
       </c>
       <c r="X50" t="n">
-        <v>314.6577570050235</v>
+        <v>79.71351546234041</v>
       </c>
       <c r="Y50" t="n">
-        <v>5.189222954927768</v>
+        <v>64.12767286642595</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Baltica-Karelia</t>
+          <t>Baltica-Sarmatia</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Kivakka intrusion</t>
+          <t>Volyn-Dniestr-Bug intrusions B</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2443</v>
+        <v>2000</v>
       </c>
       <c r="D51" t="n">
-        <v>2438</v>
+        <v>1990</v>
       </c>
       <c r="E51" t="n">
-        <v>2448</v>
+        <v>2010</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -4832,45 +4832,45 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>30.6</v>
+        <v>27.4</v>
       </c>
       <c r="H51" t="n">
-        <v>65</v>
+        <v>50.9</v>
       </c>
       <c r="I51" t="n">
-        <v>253.7</v>
+        <v>140.4</v>
       </c>
       <c r="J51" t="n">
-        <v>-16.6</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="K51" t="n">
-        <v>7.6</v>
+        <v>12.7</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Lubnina, N., Bychkov, A.V., Tarasov, N.A., Osadchii, V.O., Miklyaeva, E.P.</t>
+          <t>Elming, S.-Ã…., Shumlyanskyy, L., Kravchenko, S., Layer, P., SÃ¶derlund, U.</t>
         </is>
       </c>
       <c r="M51" t="n">
-        <v>2438</v>
+        <v>1990</v>
       </c>
       <c r="N51" t="n">
-        <v>2448</v>
+        <v>2010</v>
       </c>
       <c r="O51" t="n">
-        <v>253.7</v>
+        <v>140.4</v>
       </c>
       <c r="P51" t="n">
-        <v>-16.6</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="Q51" t="n">
-        <v>7.6</v>
+        <v>12.7</v>
       </c>
       <c r="R51" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="S51" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="T51" t="inlineStr">
         <is>
@@ -4884,34 +4884,34 @@
         <v>28</v>
       </c>
       <c r="W51" t="n">
-        <v>-33.37935846433284</v>
+        <v>47.5937405245742</v>
       </c>
       <c r="X51" t="n">
-        <v>304.7799130100032</v>
+        <v>36.32525271172614</v>
       </c>
       <c r="Y51" t="n">
-        <v>-52.80569857324302</v>
+        <v>65.45557791819445</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Baltica-Karelia</t>
+          <t>Baltica-Kola</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Karelian Dykes</t>
+          <t>Kuetsyarvi Formation</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2446</v>
+        <v>2060</v>
       </c>
       <c r="D52" t="n">
-        <v>2441</v>
+        <v>2052</v>
       </c>
       <c r="E52" t="n">
-        <v>2451</v>
+        <v>2068</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -4919,45 +4919,45 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>30.700001</v>
+        <v>29.5</v>
       </c>
       <c r="H52" t="n">
-        <v>66</v>
+        <v>69.5</v>
       </c>
       <c r="I52" t="n">
-        <v>278.700012</v>
+        <v>300.8</v>
       </c>
       <c r="J52" t="n">
-        <v>-19.9</v>
+        <v>24.7</v>
       </c>
       <c r="K52" t="n">
-        <v>6.1</v>
+        <v>16.40426774</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Mertanen,S., Halls,H.C., Vuollo,J.I., Pesonen,L.J., Stepanov,V.S.</t>
+          <t>Torsvik, T.H. and Meert, J.</t>
         </is>
       </c>
       <c r="M52" t="n">
-        <v>2441</v>
+        <v>2052</v>
       </c>
       <c r="N52" t="n">
-        <v>2451</v>
+        <v>2068</v>
       </c>
       <c r="O52" t="n">
-        <v>278.700012</v>
+        <v>300.8</v>
       </c>
       <c r="P52" t="n">
-        <v>-19.9</v>
+        <v>24.7</v>
       </c>
       <c r="Q52" t="n">
-        <v>6.1</v>
+        <v>16.40426774</v>
       </c>
       <c r="R52" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="S52" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="T52" t="inlineStr">
         <is>
@@ -4971,34 +4971,34 @@
         <v>28</v>
       </c>
       <c r="W52" t="n">
-        <v>-26.24225641196026</v>
+        <v>23.26794062335917</v>
       </c>
       <c r="X52" t="n">
-        <v>278.3410330941796</v>
+        <v>278.9735268919012</v>
       </c>
       <c r="Y52" t="n">
-        <v>-44.59479684877332</v>
+        <v>40.69585227923566</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Baltica-Karelia</t>
+          <t>Baltica-Sarmatia</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Mean D Burakovskaya intrusion and remagnetized Avdeev/Shalskiy dykes</t>
+          <t>Volyn-Dniestr-Bug intrusions A-group</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2449</v>
+        <v>2061</v>
       </c>
       <c r="D53" t="n">
-        <v>2448</v>
+        <v>2041</v>
       </c>
       <c r="E53" t="n">
-        <v>2450</v>
+        <v>2081</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -5006,45 +5006,45 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>36.05</v>
+        <v>29.8</v>
       </c>
       <c r="H53" t="n">
-        <v>61.94</v>
+        <v>49.6</v>
       </c>
       <c r="I53" t="n">
-        <v>68.5</v>
+        <v>182.9</v>
       </c>
       <c r="J53" t="n">
-        <v>14.3</v>
+        <v>15.7</v>
       </c>
       <c r="K53" t="n">
-        <v>9.279547403</v>
+        <v>13.7</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Sherbakova et al 2017; Mertanen, S., Vuollo, J.I., Huhma, H., Arestova N.A., Kovalenko, A.</t>
+          <t>Elming, S.-Ã…., Shumlyanskyy, L., Kravchenko, S., Layer, P., SÃ¶derlund, U.</t>
         </is>
       </c>
       <c r="M53" t="n">
-        <v>2448</v>
+        <v>2041</v>
       </c>
       <c r="N53" t="n">
-        <v>2450</v>
+        <v>2081</v>
       </c>
       <c r="O53" t="n">
-        <v>68.5</v>
+        <v>182.9</v>
       </c>
       <c r="P53" t="n">
-        <v>14.3</v>
+        <v>15.7</v>
       </c>
       <c r="Q53" t="n">
-        <v>9.279547403</v>
+        <v>13.7</v>
       </c>
       <c r="R53" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="S53" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -5058,13 +5058,13 @@
         <v>28</v>
       </c>
       <c r="W53" t="n">
-        <v>33.02555064791223</v>
+        <v>-7.987132944778764</v>
       </c>
       <c r="X53" t="n">
-        <v>131.3574545725372</v>
+        <v>24.35402788229668</v>
       </c>
       <c r="Y53" t="n">
-        <v>52.43318800652726</v>
+        <v>-15.67537676742309</v>
       </c>
     </row>
     <row r="54">
@@ -5075,17 +5075,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Mean D' Shalskiy-Deda-Gorelyi-Glubokaya dyke</t>
+          <t>Varpaisjärvi dolerites &amp; basement</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2511</v>
+        <v>2295</v>
       </c>
       <c r="D54" t="n">
-        <v>2448</v>
+        <v>2290</v>
       </c>
       <c r="E54" t="n">
-        <v>2512</v>
+        <v>2300</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -5093,45 +5093,45 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>36.05</v>
+        <v>27.8</v>
       </c>
       <c r="H54" t="n">
-        <v>61.94</v>
+        <v>63.4</v>
       </c>
       <c r="I54" t="n">
-        <v>221.9</v>
+        <v>262.3</v>
       </c>
       <c r="J54" t="n">
-        <v>26.2</v>
+        <v>-17.4</v>
       </c>
       <c r="K54" t="n">
-        <v>4.949747468</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Sherbakova et al 2017; Mertanen, S., Vuollo, J.I., Huhma, H., Arestova N.A., Kovalenko, A.</t>
+          <t>Mertanen, S., Hölttä, P., Pesonen, L.J., Paavola, J.,</t>
         </is>
       </c>
       <c r="M54" t="n">
-        <v>2448</v>
+        <v>2290</v>
       </c>
       <c r="N54" t="n">
-        <v>2512</v>
+        <v>2300</v>
       </c>
       <c r="O54" t="n">
-        <v>221.9</v>
+        <v>262.3</v>
       </c>
       <c r="P54" t="n">
-        <v>26.2</v>
+        <v>-17.4</v>
       </c>
       <c r="Q54" t="n">
-        <v>4.949747468</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="R54" t="n">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="S54" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="T54" t="inlineStr">
         <is>
@@ -5145,80 +5145,80 @@
         <v>28</v>
       </c>
       <c r="W54" t="n">
-        <v>0.8599732743229822</v>
+        <v>-30.85572545050428</v>
       </c>
       <c r="X54" t="n">
-        <v>347.5509769073457</v>
+        <v>295.4863304832984</v>
       </c>
       <c r="Y54" t="n">
-        <v>1.71955925178357</v>
+        <v>-50.07383311007023</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Baltica-Kola</t>
+          <t>Baltica-Karelia</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Tsuomasvarri Gabbro-Diorite Intrusion</t>
+          <t>Taivalkoski 2.3 Ga dyke</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1931</v>
+        <v>2339</v>
       </c>
       <c r="D55" t="n">
-        <v>1929</v>
+        <v>2321</v>
       </c>
       <c r="E55" t="n">
-        <v>1933</v>
+        <v>2357</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="G55" t="n">
-        <v>28.299999</v>
+        <v>28.1</v>
       </c>
       <c r="H55" t="n">
-        <v>69.900002</v>
+        <v>65.5</v>
       </c>
       <c r="I55" t="n">
-        <v>247.300003</v>
+        <v>257.3</v>
       </c>
       <c r="J55" t="n">
-        <v>40.200001</v>
+        <v>20.4</v>
       </c>
       <c r="K55" t="n">
-        <v>6.015812497</v>
+        <v>6.3</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Mertanen,S., Pesonen,L.J.</t>
+          <t>Salminen, J., Halls, H.C., Mertanen, S., Pesonen, L.J., Vuollo, J., SÃ¶derlund, U.</t>
         </is>
       </c>
       <c r="M55" t="n">
-        <v>1929</v>
+        <v>2321</v>
       </c>
       <c r="N55" t="n">
-        <v>1933</v>
+        <v>2357</v>
       </c>
       <c r="O55" t="n">
-        <v>247.300003</v>
+        <v>257.3</v>
       </c>
       <c r="P55" t="n">
-        <v>40.200001</v>
+        <v>20.4</v>
       </c>
       <c r="Q55" t="n">
-        <v>6.015812497</v>
+        <v>6.3</v>
       </c>
       <c r="R55" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="S55" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="T55" t="inlineStr">
         <is>
@@ -5232,34 +5232,34 @@
         <v>28</v>
       </c>
       <c r="W55" t="n">
-        <v>18.72532451752087</v>
+        <v>2.599943141397745</v>
       </c>
       <c r="X55" t="n">
-        <v>329.2820768653556</v>
+        <v>314.6577570050235</v>
       </c>
       <c r="Y55" t="n">
-        <v>34.13523227034082</v>
+        <v>5.189222954927768</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Baltica-Kola</t>
+          <t>Baltica-Karelia</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Kuetsyarvi Formation</t>
+          <t>Kivakka intrusion</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2060</v>
+        <v>2443</v>
       </c>
       <c r="D56" t="n">
-        <v>2052</v>
+        <v>2438</v>
       </c>
       <c r="E56" t="n">
-        <v>2068</v>
+        <v>2448</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -5267,45 +5267,45 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>29.5</v>
+        <v>30.6</v>
       </c>
       <c r="H56" t="n">
-        <v>69.5</v>
+        <v>65</v>
       </c>
       <c r="I56" t="n">
-        <v>300.8</v>
+        <v>253.7</v>
       </c>
       <c r="J56" t="n">
-        <v>24.7</v>
+        <v>-16.6</v>
       </c>
       <c r="K56" t="n">
-        <v>16.40426774</v>
+        <v>7.6</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Torsvik, T.H. and Meert, J.</t>
+          <t>Lubnina, N., Bychkov, A.V., Tarasov, N.A., Osadchii, V.O., Miklyaeva, E.P.</t>
         </is>
       </c>
       <c r="M56" t="n">
-        <v>2052</v>
+        <v>2438</v>
       </c>
       <c r="N56" t="n">
-        <v>2068</v>
+        <v>2448</v>
       </c>
       <c r="O56" t="n">
-        <v>300.8</v>
+        <v>253.7</v>
       </c>
       <c r="P56" t="n">
-        <v>24.7</v>
+        <v>-16.6</v>
       </c>
       <c r="Q56" t="n">
-        <v>16.40426774</v>
+        <v>7.6</v>
       </c>
       <c r="R56" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="S56" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="T56" t="inlineStr">
         <is>
@@ -5319,34 +5319,34 @@
         <v>28</v>
       </c>
       <c r="W56" t="n">
-        <v>23.26794062335917</v>
+        <v>-33.37935846433284</v>
       </c>
       <c r="X56" t="n">
-        <v>278.9735268919012</v>
+        <v>304.7799130100032</v>
       </c>
       <c r="Y56" t="n">
-        <v>40.69585227923566</v>
+        <v>-52.80569857324302</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Baltica-Sarmatia</t>
+          <t>Baltica-Karelia</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Volyn-Dniestr-Bug intrusions E</t>
+          <t>Karelian Dykes</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1722</v>
+        <v>2446</v>
       </c>
       <c r="D57" t="n">
-        <v>1710</v>
+        <v>2441</v>
       </c>
       <c r="E57" t="n">
-        <v>1734</v>
+        <v>2451</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -5354,45 +5354,45 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>29.6</v>
+        <v>30.700001</v>
       </c>
       <c r="H57" t="n">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="I57" t="n">
-        <v>163.2</v>
+        <v>278.700012</v>
       </c>
       <c r="J57" t="n">
-        <v>10.7</v>
+        <v>-19.9</v>
       </c>
       <c r="K57" t="n">
-        <v>10.2</v>
+        <v>6.1</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Elming, S.-Ã…., Shumlyanskyy, L., Kravchenko, S., Layer, P., SÃ¶derlund, U.</t>
+          <t>Mertanen,S., Halls,H.C., Vuollo,J.I., Pesonen,L.J., Stepanov,V.S.</t>
         </is>
       </c>
       <c r="M57" t="n">
-        <v>1710</v>
+        <v>2441</v>
       </c>
       <c r="N57" t="n">
-        <v>1734</v>
+        <v>2451</v>
       </c>
       <c r="O57" t="n">
-        <v>163.2</v>
+        <v>278.700012</v>
       </c>
       <c r="P57" t="n">
-        <v>10.7</v>
+        <v>-19.9</v>
       </c>
       <c r="Q57" t="n">
-        <v>10.2</v>
+        <v>6.1</v>
       </c>
       <c r="R57" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="S57" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="T57" t="inlineStr">
         <is>
@@ -5406,80 +5406,80 @@
         <v>28</v>
       </c>
       <c r="W57" t="n">
-        <v>-7.976730154751991</v>
+        <v>-26.24225641196026</v>
       </c>
       <c r="X57" t="n">
-        <v>44.35862235901306</v>
+        <v>278.3410330941796</v>
       </c>
       <c r="Y57" t="n">
-        <v>-15.65570891331447</v>
+        <v>-44.59479684877332</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Baltica-Sarmatia</t>
+          <t>Baltica-Karelia</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Volyn-Dniestr-Bug intrusions C+D</t>
+          <t>Mean D Burakovskaya intrusion and remagnetized Avdeev/Shalskiy dykes</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1755</v>
+        <v>2449</v>
       </c>
       <c r="D58" t="n">
-        <v>1740</v>
+        <v>2448</v>
       </c>
       <c r="E58" t="n">
-        <v>1770</v>
+        <v>2450</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>28.6</v>
+        <v>36.05</v>
       </c>
       <c r="H58" t="n">
-        <v>50.6</v>
+        <v>61.94</v>
       </c>
       <c r="I58" t="n">
-        <v>169.1</v>
+        <v>68.5</v>
       </c>
       <c r="J58" t="n">
-        <v>26.5</v>
+        <v>14.3</v>
       </c>
       <c r="K58" t="n">
-        <v>3.9</v>
+        <v>9.279547403</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Elming, S.-Ã…., Shumlyanskyy, L., Kravchenko, S., Layer, P., SÃ¶derlund, U.</t>
+          <t>Sherbakova et al 2017; Mertanen, S., Vuollo, J.I., Huhma, H., Arestova N.A., Kovalenko, A.</t>
         </is>
       </c>
       <c r="M58" t="n">
-        <v>1740</v>
+        <v>2448</v>
       </c>
       <c r="N58" t="n">
-        <v>1770</v>
+        <v>2450</v>
       </c>
       <c r="O58" t="n">
-        <v>169.1</v>
+        <v>68.5</v>
       </c>
       <c r="P58" t="n">
-        <v>26.5</v>
+        <v>14.3</v>
       </c>
       <c r="Q58" t="n">
-        <v>3.9</v>
+        <v>9.279547403</v>
       </c>
       <c r="R58" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="S58" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
@@ -5493,34 +5493,34 @@
         <v>28</v>
       </c>
       <c r="W58" t="n">
-        <v>5.493033338051561</v>
+        <v>33.02555064791223</v>
       </c>
       <c r="X58" t="n">
-        <v>34.37301626167139</v>
+        <v>131.3574545725372</v>
       </c>
       <c r="Y58" t="n">
-        <v>10.88690669551862</v>
+        <v>52.43318800652726</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Baltica-Sarmatia</t>
+          <t>Baltica-Karelia</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Volyn-Dniestr-Bug intrusions B</t>
+          <t>Mean D' Shalskiy-Deda-Gorelyi-Glubokaya dyke</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2000</v>
+        <v>2511</v>
       </c>
       <c r="D59" t="n">
-        <v>1990</v>
+        <v>2448</v>
       </c>
       <c r="E59" t="n">
-        <v>2010</v>
+        <v>2512</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -5528,45 +5528,45 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>27.4</v>
+        <v>36.05</v>
       </c>
       <c r="H59" t="n">
-        <v>50.9</v>
+        <v>61.94</v>
       </c>
       <c r="I59" t="n">
-        <v>140.4</v>
+        <v>221.9</v>
       </c>
       <c r="J59" t="n">
-        <v>64.40000000000001</v>
+        <v>26.2</v>
       </c>
       <c r="K59" t="n">
-        <v>12.7</v>
+        <v>4.949747468</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Elming, S.-Ã…., Shumlyanskyy, L., Kravchenko, S., Layer, P., SÃ¶derlund, U.</t>
+          <t>Sherbakova et al 2017; Mertanen, S., Vuollo, J.I., Huhma, H., Arestova N.A., Kovalenko, A.</t>
         </is>
       </c>
       <c r="M59" t="n">
-        <v>1990</v>
+        <v>2448</v>
       </c>
       <c r="N59" t="n">
-        <v>2010</v>
+        <v>2512</v>
       </c>
       <c r="O59" t="n">
-        <v>140.4</v>
+        <v>221.9</v>
       </c>
       <c r="P59" t="n">
-        <v>64.40000000000001</v>
+        <v>26.2</v>
       </c>
       <c r="Q59" t="n">
-        <v>12.7</v>
+        <v>4.949747468</v>
       </c>
       <c r="R59" t="n">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="S59" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="T59" t="inlineStr">
         <is>
@@ -5580,100 +5580,13 @@
         <v>28</v>
       </c>
       <c r="W59" t="n">
-        <v>47.5937405245742</v>
+        <v>0.8599732743229822</v>
       </c>
       <c r="X59" t="n">
-        <v>36.32525271172614</v>
+        <v>347.5509769073457</v>
       </c>
       <c r="Y59" t="n">
-        <v>65.45557791819445</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Baltica-Sarmatia</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Volyn-Dniestr-Bug intrusions A-group</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>2061</v>
-      </c>
-      <c r="D60" t="n">
-        <v>2041</v>
-      </c>
-      <c r="E60" t="n">
-        <v>2081</v>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G60" t="n">
-        <v>29.8</v>
-      </c>
-      <c r="H60" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="I60" t="n">
-        <v>182.9</v>
-      </c>
-      <c r="J60" t="n">
-        <v>15.7</v>
-      </c>
-      <c r="K60" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>Elming, S.-Ã…., Shumlyanskyy, L., Kravchenko, S., Layer, P., SÃ¶derlund, U.</t>
-        </is>
-      </c>
-      <c r="M60" t="n">
-        <v>2041</v>
-      </c>
-      <c r="N60" t="n">
-        <v>2081</v>
-      </c>
-      <c r="O60" t="n">
-        <v>182.9</v>
-      </c>
-      <c r="P60" t="n">
-        <v>15.7</v>
-      </c>
-      <c r="Q60" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="R60" t="n">
-        <v>20</v>
-      </c>
-      <c r="S60" t="n">
-        <v>20</v>
-      </c>
-      <c r="T60" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="U60" t="n">
-        <v>64</v>
-      </c>
-      <c r="V60" t="n">
-        <v>28</v>
-      </c>
-      <c r="W60" t="n">
-        <v>-7.987132944778764</v>
-      </c>
-      <c r="X60" t="n">
-        <v>24.35402788229668</v>
-      </c>
-      <c r="Y60" t="n">
-        <v>-15.67537676742309</v>
+        <v>1.71955925178357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>